<commit_message>
WIP (task190, task202): a repair mid-rebuild and a generator being written, committed for durability
Not a status change. task190's repair pass rewrote its checks, documents, verifier, figures.json, goldens
and metadata within the last minute and is mid-rebuild, so its ask figures have moved by design while the
main call's figures are the thing I will check at hand-back. task202's builder now has eight generator
modules. Neither is gate-checked here.

Committed because the container is ephemeral. The real status commits follow when each hands back and the
gates have been re-run on the shipped bytes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task190/golden/recovery_attainment_2026.xlsx
+++ b/task190/golden/recovery_attainment_2026.xlsx
@@ -1275,10 +1275,10 @@
         <v>32.54</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>16.66</v>
+        <v>16.53</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
WIP (task190): the ask re-siting mid-rebuild, committed for durability
Not a status change. task190's ask rework touched its ceiling model, figures and golden workbook a minute
before this commit and is mid-rebuild, so its ask figures are moving by design while the call's figures are
what I check at hand-back. Not gate-checked here. Committed because the container is ephemeral.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task190/golden/recovery_attainment_2026.xlsx
+++ b/task190/golden/recovery_attainment_2026.xlsx
@@ -1224,22 +1224,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Collection round 2026: field effort by regional team</t>
+          <t>Collection round 2026: contacts by region of the enterprise contacted</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Field days are counted once per field visit; a visit covers several enterprises. Usable returns are counted once per collection case.</t>
+          <t>A case sits in the region of the enterprise it was opened for, which is the holder of its permit number over the round and not always the holder of record now. Contacts and usable returns are counted once.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Field days consumed</t>
+          <t>Contacts made</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Usable returns per field day</t>
+          <t>Contacts per usable return</t>
         </is>
       </c>
     </row>
@@ -1271,14 +1271,14 @@
           <t>Norte</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>32.54</v>
+      <c r="B5" s="10" t="n">
+        <v>1965</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>538</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>16.53</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="6">
@@ -1287,14 +1287,14 @@
           <t>Centro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>25.69</v>
+      <c r="B6" s="10" t="n">
+        <v>1387</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>381</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>14.83</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="7">
@@ -1303,14 +1303,14 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>29.8</v>
+      <c r="B7" s="10" t="n">
+        <v>1652</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>430</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>14.43</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="8">
@@ -1319,14 +1319,14 @@
           <t>Alentejo</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
-        <v>10.11</v>
+      <c r="B8" s="10" t="n">
+        <v>641</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>166</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>16.42</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="9">
@@ -1335,14 +1335,14 @@
           <t>Algarve</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
-        <v>7.66</v>
+      <c r="B9" s="10" t="n">
+        <v>434</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>115</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>15.01</v>
+        <v>3.77</v>
       </c>
     </row>
   </sheetData>
@@ -1493,7 +1493,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Receipts are on a receipt-date basis and attributed to the region of collection.</t>
+          <t>Receipts are on a receipt-date basis and attributed to the region of collection. A municipality's collections are its own return for the year, taken once.</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1731,46 +1731,58 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Field day</t>
+          <t>Collection case</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>eight hours, as the survey's collection documentation books it; the response log's time_unit column gives the unit each row is recorded in</t>
+          <t>one per enterprise issued, in the region of the enterprise the case was opened for; the response log carries the permit number the case was opened under and the crosswalk is effective dated</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Rounding</t>
+          <t>Municipal collections</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>rates, shortfalls and shares to one decimal, tonnages to the nearest tonne, field days and returns per day to two decimals</t>
+          <t>each municipality's own return, counted once; the inter-municipal associations report for their members</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
+          <t>Rounding</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>rates, shortfalls and shares to one decimal, tonnages to the nearest tonne, contacts to the nearest whole and contacts per usable return to two decimals</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
           <t>Standard error</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>of the recovery rate, shown for working; the plan reports attainment without a precision measure</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Business Waste Survey and the National Waste Movement Register</t>
         </is>

</xml_diff>